<commit_message>
Updated few scripts- Added a new project path in json file to trigger TP's
</commit_message>
<xml_diff>
--- a/uploads/NewFileLoanPopVerification.xlsx
+++ b/uploads/NewFileLoanPopVerification.xlsx
@@ -540,7 +540,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>TestSigma_10-04-2026_SC1_ct_309</v>
+        <v>TestSigma_20-04-2026_SC1_0r_376</v>
       </c>
       <c r="B2" s="1">
         <v>2001</v>
@@ -654,7 +654,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>TestSigma_10-04-2026_SC1_fv_722</v>
+        <v>TestSigma_20-04-2026_SC1_pr_214</v>
       </c>
       <c r="B3" s="1">
         <v>2001</v>
@@ -768,7 +768,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="str">
-        <v>TestSigma_10-04-2026_SC1_dq_425</v>
+        <v>TestSigma_20-04-2026_SC1_5d_940</v>
       </c>
       <c r="B4" s="1">
         <v>2001</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="str">
-        <v>TestSigma_10-04-2026_SC1_4y_170</v>
+        <v>TestSigma_20-04-2026_SC1_vm_975</v>
       </c>
       <c r="B5" s="1">
         <v>2001</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="str">
-        <v>TestSigma_10-04-2026_SC1_13_877</v>
+        <v>TestSigma_20-04-2026_SC1_7x_243</v>
       </c>
       <c r="B6" s="1">
         <v>2001</v>

</xml_diff>